<commit_message>
Ajuste script de partidas
</commit_message>
<xml_diff>
--- a/Planilhas/BPs.xlsx
+++ b/Planilhas/BPs.xlsx
@@ -1,31 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\python_scripts\PLANILHAS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F278032-8D4C-43CA-9C50-7DF5754E3222}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFD1D28F-8CF6-4B4D-B08C-82336AAB6E1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28635" yWindow="-135" windowWidth="29130" windowHeight="15810" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="201">
   <si>
     <t>BP</t>
   </si>
@@ -34,6 +45,600 @@
   </si>
   <si>
     <t>EMAIL</t>
+  </si>
+  <si>
+    <t>35999207208</t>
+  </si>
+  <si>
+    <t>35991222086</t>
+  </si>
+  <si>
+    <t>35997506822</t>
+  </si>
+  <si>
+    <t>35988836248</t>
+  </si>
+  <si>
+    <t>35988347938</t>
+  </si>
+  <si>
+    <t>35991168177</t>
+  </si>
+  <si>
+    <t>35984516476</t>
+  </si>
+  <si>
+    <t>35999533290</t>
+  </si>
+  <si>
+    <t>35998897922</t>
+  </si>
+  <si>
+    <t>35988359251</t>
+  </si>
+  <si>
+    <t>35984051453</t>
+  </si>
+  <si>
+    <t>35998545432</t>
+  </si>
+  <si>
+    <t>82991417394</t>
+  </si>
+  <si>
+    <t>35998830370</t>
+  </si>
+  <si>
+    <t>35988649350</t>
+  </si>
+  <si>
+    <t>35987092307</t>
+  </si>
+  <si>
+    <t>35991247016</t>
+  </si>
+  <si>
+    <t>35999440334</t>
+  </si>
+  <si>
+    <t>35999539600</t>
+  </si>
+  <si>
+    <t>35988665169</t>
+  </si>
+  <si>
+    <t>35988849041</t>
+  </si>
+  <si>
+    <t>0001005615</t>
+  </si>
+  <si>
+    <t>3799312276</t>
+  </si>
+  <si>
+    <t>adrestaurantedouradao@yahoo.com.br</t>
+  </si>
+  <si>
+    <t>0001005661</t>
+  </si>
+  <si>
+    <t>3734213737</t>
+  </si>
+  <si>
+    <t>taquinholuz@hotmail.com</t>
+  </si>
+  <si>
+    <t>0001006779</t>
+  </si>
+  <si>
+    <t>3798404251</t>
+  </si>
+  <si>
+    <t>merceariatremnosso@gmail.com</t>
+  </si>
+  <si>
+    <t>0001007630</t>
+  </si>
+  <si>
+    <t>3791372612</t>
+  </si>
+  <si>
+    <t>mariaarauj775@gmail.com</t>
+  </si>
+  <si>
+    <t>0001007681</t>
+  </si>
+  <si>
+    <t>3799296023</t>
+  </si>
+  <si>
+    <t>silviaapsantos367@gmail.com</t>
+  </si>
+  <si>
+    <t>0001007713</t>
+  </si>
+  <si>
+    <t>34998406873</t>
+  </si>
+  <si>
+    <t>restaurantegameleira@hotmail.com</t>
+  </si>
+  <si>
+    <t>0001007934</t>
+  </si>
+  <si>
+    <t>3799428524</t>
+  </si>
+  <si>
+    <t>jeangermanomaumau@yahoo.com.br</t>
+  </si>
+  <si>
+    <t>0001008230</t>
+  </si>
+  <si>
+    <t>3798223434</t>
+  </si>
+  <si>
+    <t>maurotrigo@yahoo.com</t>
+  </si>
+  <si>
+    <t>0001009975</t>
+  </si>
+  <si>
+    <t>3193455441</t>
+  </si>
+  <si>
+    <t>superbarataoluz@gmail.com</t>
+  </si>
+  <si>
+    <t>0001012159</t>
+  </si>
+  <si>
+    <t>3734311339</t>
+  </si>
+  <si>
+    <t>supermercadonoe@gmail.com</t>
+  </si>
+  <si>
+    <t>0001012217</t>
+  </si>
+  <si>
+    <t>3733532061</t>
+  </si>
+  <si>
+    <t>rinaldocont@netsite.com.br</t>
+  </si>
+  <si>
+    <t>0001012224</t>
+  </si>
+  <si>
+    <t>3799998977</t>
+  </si>
+  <si>
+    <t>merceariabrito@yahoo.com</t>
+  </si>
+  <si>
+    <t>0001013780</t>
+  </si>
+  <si>
+    <t>3791170129</t>
+  </si>
+  <si>
+    <t>ray-seixas@hotmail.com</t>
+  </si>
+  <si>
+    <t>0001014102</t>
+  </si>
+  <si>
+    <t>3734311412</t>
+  </si>
+  <si>
+    <t>supermercadosaopedroacg@yahoo.com.br</t>
+  </si>
+  <si>
+    <t>0001014103</t>
+  </si>
+  <si>
+    <t>313072050</t>
+  </si>
+  <si>
+    <t>avenidarestaurante1@gmail.com</t>
+  </si>
+  <si>
+    <t>0001014106</t>
+  </si>
+  <si>
+    <t>3734314223</t>
+  </si>
+  <si>
+    <t>supermercadoisrael@hotmail.com</t>
+  </si>
+  <si>
+    <t>0001014153</t>
+  </si>
+  <si>
+    <t>3734211535</t>
+  </si>
+  <si>
+    <t>total_supermercado@hotmail.com</t>
+  </si>
+  <si>
+    <t>0001016351</t>
+  </si>
+  <si>
+    <t>3734212434</t>
+  </si>
+  <si>
+    <t>lucianarestfogao@gmail.com</t>
+  </si>
+  <si>
+    <t>0001017475</t>
+  </si>
+  <si>
+    <t>3798321958</t>
+  </si>
+  <si>
+    <t>elisneicatielisilvaolherolher@gmail.com</t>
+  </si>
+  <si>
+    <t>0001017572</t>
+  </si>
+  <si>
+    <t>3798429841</t>
+  </si>
+  <si>
+    <t>elielmacedo311@gmail.com</t>
+  </si>
+  <si>
+    <t>0001017793</t>
+  </si>
+  <si>
+    <t>3734311744</t>
+  </si>
+  <si>
+    <t>gelsonga76@gmail.com</t>
+  </si>
+  <si>
+    <t>0001018650</t>
+  </si>
+  <si>
+    <t>3788441494</t>
+  </si>
+  <si>
+    <t>vicentedepaula220570@gmail.com</t>
+  </si>
+  <si>
+    <t>0001019181</t>
+  </si>
+  <si>
+    <t>3796712551</t>
+  </si>
+  <si>
+    <t>valdirromualdokz@gmail.com</t>
+  </si>
+  <si>
+    <t>0001019344</t>
+  </si>
+  <si>
+    <t>3799414111</t>
+  </si>
+  <si>
+    <t>restaurantegarrafinha123@gmail.com</t>
+  </si>
+  <si>
+    <t>0001020012</t>
+  </si>
+  <si>
+    <t>3798226634</t>
+  </si>
+  <si>
+    <t>bhrendaingridy83@gmail.com</t>
+  </si>
+  <si>
+    <t>0001020183</t>
+  </si>
+  <si>
+    <t>3188374459</t>
+  </si>
+  <si>
+    <t>juridico1@topcontroller.com.br</t>
+  </si>
+  <si>
+    <t>0001020499</t>
+  </si>
+  <si>
+    <t>3798627313</t>
+  </si>
+  <si>
+    <t>breno@suportecontabilidade.com.br</t>
+  </si>
+  <si>
+    <t>0001021470</t>
+  </si>
+  <si>
+    <t>3799129335</t>
+  </si>
+  <si>
+    <t>luannamarinsvieiracampos21@gmail.com</t>
+  </si>
+  <si>
+    <t>0001023103</t>
+  </si>
+  <si>
+    <t>3796704875</t>
+  </si>
+  <si>
+    <t>vanessafatima199@gmail.com</t>
+  </si>
+  <si>
+    <t>0001023819</t>
+  </si>
+  <si>
+    <t>3798221004</t>
+  </si>
+  <si>
+    <t>zequinhavictor@gmail.com</t>
+  </si>
+  <si>
+    <t>0001024548</t>
+  </si>
+  <si>
+    <t>3799351975</t>
+  </si>
+  <si>
+    <t>jeffersonwallacejacobteodoro@gmail.com</t>
+  </si>
+  <si>
+    <t>0001026115</t>
+  </si>
+  <si>
+    <t>3799488759</t>
+  </si>
+  <si>
+    <t>geysieneferreira29@gmail.com</t>
+  </si>
+  <si>
+    <t>0001026118</t>
+  </si>
+  <si>
+    <t>3788442375</t>
+  </si>
+  <si>
+    <t>rickguimaraes@live.com</t>
+  </si>
+  <si>
+    <t>0001026367</t>
+  </si>
+  <si>
+    <t>3799196085</t>
+  </si>
+  <si>
+    <t>matheusaurelio-2010@hotmail.com</t>
+  </si>
+  <si>
+    <t>0001027699</t>
+  </si>
+  <si>
+    <t>3788446566</t>
+  </si>
+  <si>
+    <t>onofrefaria@123yahoo.com.br</t>
+  </si>
+  <si>
+    <t>0001027982</t>
+  </si>
+  <si>
+    <t>3734213010</t>
+  </si>
+  <si>
+    <t>cd@postocaxuxa.com.br</t>
+  </si>
+  <si>
+    <t>0001028733</t>
+  </si>
+  <si>
+    <t>3799358377</t>
+  </si>
+  <si>
+    <t>pegomarcia18@gmail.com</t>
+  </si>
+  <si>
+    <t>0001028857</t>
+  </si>
+  <si>
+    <t>3734241096</t>
+  </si>
+  <si>
+    <t>rosenirbencardoso@gmail.com</t>
+  </si>
+  <si>
+    <t>0001028863</t>
+  </si>
+  <si>
+    <t>3799254542</t>
+  </si>
+  <si>
+    <t>mercdopopular@gmail.com</t>
+  </si>
+  <si>
+    <t>0001028877</t>
+  </si>
+  <si>
+    <t>3799868958</t>
+  </si>
+  <si>
+    <t>sandrolpatinho@gmail.com</t>
+  </si>
+  <si>
+    <t>0001029835</t>
+  </si>
+  <si>
+    <t>37999695949</t>
+  </si>
+  <si>
+    <t>camillaccbbss@hotmail.com</t>
+  </si>
+  <si>
+    <t>0001030065</t>
+  </si>
+  <si>
+    <t>37999769066</t>
+  </si>
+  <si>
+    <t>neymarcaetanojhow@hotmail.com</t>
+  </si>
+  <si>
+    <t>0001030071</t>
+  </si>
+  <si>
+    <t>37991221370</t>
+  </si>
+  <si>
+    <t>edenilsonchiesa@gmail.com</t>
+  </si>
+  <si>
+    <t>0001030461</t>
+  </si>
+  <si>
+    <t>37999979142</t>
+  </si>
+  <si>
+    <t>lucasviniciustometavares@gmail.com</t>
+  </si>
+  <si>
+    <t>0001030626</t>
+  </si>
+  <si>
+    <t>37988002577</t>
+  </si>
+  <si>
+    <t>leandrocarvalho55@icloud.com</t>
+  </si>
+  <si>
+    <t>0001013954</t>
+  </si>
+  <si>
+    <t>casadecarnesnadinho@gmail.com</t>
+  </si>
+  <si>
+    <t>0001028663</t>
+  </si>
+  <si>
+    <t>veronikajm1011@gmail.com</t>
+  </si>
+  <si>
+    <t>0001023985</t>
+  </si>
+  <si>
+    <t>sararizialino@gmail.com</t>
+  </si>
+  <si>
+    <t>0001006957</t>
+  </si>
+  <si>
+    <t>abreuabreuroulien@gmail.com</t>
+  </si>
+  <si>
+    <t>0001028580</t>
+  </si>
+  <si>
+    <t>roselucas141@gmail.com</t>
+  </si>
+  <si>
+    <t>0001019055</t>
+  </si>
+  <si>
+    <t>gesmobar64@gmail.com</t>
+  </si>
+  <si>
+    <t>0001012227</t>
+  </si>
+  <si>
+    <t>alinejulieder@gmail.com</t>
+  </si>
+  <si>
+    <t>0001030046</t>
+  </si>
+  <si>
+    <t>sebastiana2024justino@mail.com</t>
+  </si>
+  <si>
+    <t>0001005854</t>
+  </si>
+  <si>
+    <t>isadoramartinsalves@gmail.com</t>
+  </si>
+  <si>
+    <t>0001028675</t>
+  </si>
+  <si>
+    <t>merceariasaovicentelavras@gmail.com</t>
+  </si>
+  <si>
+    <t>0001028698</t>
+  </si>
+  <si>
+    <t>jcsv2016@outlook.com</t>
+  </si>
+  <si>
+    <t>0001030319</t>
+  </si>
+  <si>
+    <t>rodriguesantonioadelino@gmail.com</t>
+  </si>
+  <si>
+    <t>0001028892</t>
+  </si>
+  <si>
+    <t>juscelino.metalar@gmail.com</t>
+  </si>
+  <si>
+    <t>0001024253</t>
+  </si>
+  <si>
+    <t>patricianatalina21@gmail.com</t>
+  </si>
+  <si>
+    <t>0001012799</t>
+  </si>
+  <si>
+    <t>roseandre68@gmail.com</t>
+  </si>
+  <si>
+    <t>0001027475</t>
+  </si>
+  <si>
+    <t>ljpereira2013@gmail.com</t>
+  </si>
+  <si>
+    <t>0001015160</t>
+  </si>
+  <si>
+    <t>mesquita@navinet.com.br</t>
+  </si>
+  <si>
+    <t>0001009743</t>
+  </si>
+  <si>
+    <t>vanderlei.r.tst@gmail.com</t>
+  </si>
+  <si>
+    <t>0001021226</t>
+  </si>
+  <si>
+    <t>francisetaisa@gmail.com</t>
+  </si>
+  <si>
+    <t>0001030564</t>
+  </si>
+  <si>
+    <t>ofpontello@gmail.com</t>
+  </si>
+  <si>
+    <t>0001018598</t>
+  </si>
+  <si>
+    <t>oliveirafabio320@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -77,22 +682,31 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
     <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -108,12 +722,12 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CFCA1631-0048-4E5E-B170-87472F1B5CA8}" name="Tabela1" displayName="Tabela1" ref="A1:C2" totalsRowShown="0">
-  <autoFilter ref="A1:C2" xr:uid="{CFCA1631-0048-4E5E-B170-87472F1B5CA8}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CFCA1631-0048-4E5E-B170-87472F1B5CA8}" name="Tabela1" displayName="Tabela1" ref="A1:C67" totalsRowShown="0">
+  <autoFilter ref="A1:C67" xr:uid="{CFCA1631-0048-4E5E-B170-87472F1B5CA8}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{AACB03FA-B9F3-4B8F-8ED4-26E0E26CB943}" name="BP"/>
     <tableColumn id="2" xr3:uid="{15CE7D9D-72DF-43CB-B33C-916D72F0092C}" name="TELEFONE" dataDxfId="0"/>
-    <tableColumn id="3" xr3:uid="{DA1E5BF7-41F6-4FB2-A036-CCF76E91B795}" name="EMAIL"/>
+    <tableColumn id="3" xr3:uid="{DA1E5BF7-41F6-4FB2-A036-CCF76E91B795}" name="EMAIL" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium10" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -382,18 +996,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C67"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="7.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.36328125" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.7265625" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
@@ -401,11 +1016,729 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2">
-        <v>1004829</v>
-      </c>
-      <c r="B2" s="3">
-        <v>3733532240</v>
+      <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>45</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>48</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>51</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>57</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>60</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>63</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>66</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>69</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>72</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>75</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>78</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>81</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>84</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>87</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>90</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>93</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>96</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>99</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>102</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>105</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>108</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>111</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>114</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>117</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>120</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>123</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>126</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>129</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>132</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>135</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
+        <v>138</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>141</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>144</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>147</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="C43" s="3" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
+        <v>150</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="C44" s="3" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
+        <v>153</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="C45" s="3" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
+        <v>156</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
+        <v>159</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C47" s="3" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
+        <v>161</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
+        <v>163</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C49" s="3" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
+        <v>165</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
+        <v>167</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
+        <v>169</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C52" s="3" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A53" t="s">
+        <v>171</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C53" s="3" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A54" t="s">
+        <v>173</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C54" s="3" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
+        <v>175</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C55" s="3" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A56" t="s">
+        <v>177</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C56" s="3" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A57" t="s">
+        <v>179</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C57" s="3" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A58" t="s">
+        <v>181</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C58" s="3" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A59" t="s">
+        <v>183</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C59" s="3" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A60" t="s">
+        <v>185</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C60" s="3" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A61" t="s">
+        <v>187</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C61" s="3" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
+        <v>189</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C62" s="3" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
+        <v>191</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C63" s="3" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A64" t="s">
+        <v>193</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C64" s="3" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A65" t="s">
+        <v>195</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C65" s="3" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A66" t="s">
+        <v>197</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C66" s="3" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A67" t="s">
+        <v>199</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C67" s="3" t="s">
+        <v>200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>